<commit_message>
Reclassify weld zones: FZ +/-5 mm, HAZ 5-7.5 mm, BM >7.5 mm
Replot figure and Excel workbook with user-defined spatial zone boundaries.
Region summary is now computed from the data within each zone.
</commit_message>
<xml_diff>
--- a/microhardness_hydrogen_charging.xlsx
+++ b/microhardness_hydrogen_charging.xlsx
@@ -477,13 +477,13 @@
         <v>2.3</v>
       </c>
       <c r="E3">
-        <v>222.9</v>
+        <v>225.6</v>
       </c>
       <c r="F3">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="G3">
-        <v>5.5</v>
+        <v>8.2</v>
       </c>
     </row>
     <row r="4">
@@ -502,13 +502,13 @@
         <v>2.3</v>
       </c>
       <c r="E4">
-        <v>222.2</v>
+        <v>227.6</v>
       </c>
       <c r="F4">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="G4">
-        <v>5.5</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="5">
@@ -527,13 +527,13 @@
         <v>2.4</v>
       </c>
       <c r="E5">
-        <v>221.4</v>
+        <v>229.6</v>
       </c>
       <c r="F5">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="G5">
-        <v>5.4</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="6">
@@ -552,13 +552,13 @@
         <v>2.4</v>
       </c>
       <c r="E6">
-        <v>220.7</v>
+        <v>231.6</v>
       </c>
       <c r="F6">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="G6">
-        <v>5.4</v>
+        <v>16.3</v>
       </c>
     </row>
     <row r="7">
@@ -567,7 +567,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C7">
@@ -577,13 +577,13 @@
         <v>2.4</v>
       </c>
       <c r="E7">
-        <v>220.0</v>
+        <v>233.6</v>
       </c>
       <c r="F7">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="G7">
-        <v>5.4</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="8">
@@ -592,7 +592,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C8">
@@ -602,13 +602,13 @@
         <v>2.8</v>
       </c>
       <c r="E8">
-        <v>219.6</v>
+        <v>233.2</v>
       </c>
       <c r="F8">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="G8">
-        <v>5.4</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="9">
@@ -617,7 +617,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C9">
@@ -627,13 +627,13 @@
         <v>3.2</v>
       </c>
       <c r="E9">
-        <v>219.2</v>
+        <v>232.8</v>
       </c>
       <c r="F9">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="G9">
-        <v>5.4</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="10">
@@ -642,7 +642,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C10">
@@ -652,13 +652,13 @@
         <v>3.6</v>
       </c>
       <c r="E10">
-        <v>218.8</v>
+        <v>232.4</v>
       </c>
       <c r="F10">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="G10">
-        <v>5.4</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="11">
@@ -667,7 +667,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C11">
@@ -677,13 +677,13 @@
         <v>4.0</v>
       </c>
       <c r="E11">
-        <v>218.4</v>
+        <v>232.0</v>
       </c>
       <c r="F11">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="G11">
-        <v>5.4</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="12">
@@ -692,7 +692,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C12">
@@ -702,13 +702,13 @@
         <v>4.4</v>
       </c>
       <c r="E12">
-        <v>218.1</v>
+        <v>231.6</v>
       </c>
       <c r="F12">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="G12">
-        <v>5.4</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="13">
@@ -717,7 +717,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C13">
@@ -727,13 +727,13 @@
         <v>4.7</v>
       </c>
       <c r="E13">
-        <v>219.7</v>
+        <v>233.3</v>
       </c>
       <c r="F13">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="G13">
-        <v>5.4</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="14">
@@ -742,7 +742,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C14">
@@ -752,13 +752,13 @@
         <v>5.0</v>
       </c>
       <c r="E14">
-        <v>221.3</v>
+        <v>235.0</v>
       </c>
       <c r="F14">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="G14">
-        <v>5.4</v>
+        <v>19.1</v>
       </c>
     </row>
     <row r="15">
@@ -767,7 +767,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C15">
@@ -777,13 +777,13 @@
         <v>5.4</v>
       </c>
       <c r="E15">
-        <v>223.0</v>
+        <v>236.8</v>
       </c>
       <c r="F15">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="G15">
-        <v>5.5</v>
+        <v>19.3</v>
       </c>
     </row>
     <row r="16">
@@ -792,7 +792,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C16">
@@ -802,13 +802,13 @@
         <v>5.7</v>
       </c>
       <c r="E16">
-        <v>224.6</v>
+        <v>238.5</v>
       </c>
       <c r="F16">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G16">
-        <v>5.5</v>
+        <v>19.4</v>
       </c>
     </row>
     <row r="17">
@@ -817,7 +817,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C17">
@@ -827,13 +827,13 @@
         <v>6.0</v>
       </c>
       <c r="E17">
-        <v>226.3</v>
+        <v>240.3</v>
       </c>
       <c r="F17">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G17">
-        <v>5.6</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="18">
@@ -842,7 +842,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C18">
@@ -852,13 +852,13 @@
         <v>5.3</v>
       </c>
       <c r="E18">
-        <v>225.9</v>
+        <v>239.9</v>
       </c>
       <c r="F18">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G18">
-        <v>5.5</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="19">
@@ -867,7 +867,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C19">
@@ -877,13 +877,13 @@
         <v>4.6</v>
       </c>
       <c r="E19">
-        <v>225.6</v>
+        <v>239.6</v>
       </c>
       <c r="F19">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G19">
-        <v>5.5</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="20">
@@ -892,7 +892,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C20">
@@ -902,13 +902,13 @@
         <v>3.8</v>
       </c>
       <c r="E20">
-        <v>225.3</v>
+        <v>239.3</v>
       </c>
       <c r="F20">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G20">
-        <v>5.5</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="21">
@@ -917,7 +917,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C21">
@@ -927,13 +927,13 @@
         <v>3.1</v>
       </c>
       <c r="E21">
-        <v>225.0</v>
+        <v>239.0</v>
       </c>
       <c r="F21">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G21">
-        <v>5.5</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="22">
@@ -942,7 +942,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C22">
@@ -952,13 +952,13 @@
         <v>2.4</v>
       </c>
       <c r="E22">
-        <v>224.7</v>
+        <v>238.6</v>
       </c>
       <c r="F22">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G22">
-        <v>5.5</v>
+        <v>19.4</v>
       </c>
     </row>
     <row r="23">
@@ -967,7 +967,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C23">
@@ -977,13 +977,13 @@
         <v>3.0</v>
       </c>
       <c r="E23">
-        <v>224.9</v>
+        <v>238.9</v>
       </c>
       <c r="F23">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G23">
-        <v>5.5</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="24">
@@ -992,7 +992,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C24">
@@ -1002,13 +1002,13 @@
         <v>3.6</v>
       </c>
       <c r="E24">
-        <v>225.1</v>
+        <v>239.1</v>
       </c>
       <c r="F24">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G24">
-        <v>5.5</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="25">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C25">
@@ -1027,13 +1027,13 @@
         <v>4.3</v>
       </c>
       <c r="E25">
-        <v>225.3</v>
+        <v>239.3</v>
       </c>
       <c r="F25">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G25">
-        <v>5.5</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="26">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C26">
@@ -1052,13 +1052,13 @@
         <v>4.9</v>
       </c>
       <c r="E26">
-        <v>225.5</v>
+        <v>239.5</v>
       </c>
       <c r="F26">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G26">
-        <v>5.5</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="27">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C27">
@@ -1077,13 +1077,13 @@
         <v>5.5</v>
       </c>
       <c r="E27">
-        <v>225.7</v>
+        <v>239.7</v>
       </c>
       <c r="F27">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G27">
-        <v>5.5</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="28">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C28">
@@ -1102,13 +1102,13 @@
         <v>4.9</v>
       </c>
       <c r="E28">
-        <v>225.4</v>
+        <v>238.4</v>
       </c>
       <c r="F28">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G28">
-        <v>5.5</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="29">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C29">
@@ -1127,13 +1127,13 @@
         <v>4.3</v>
       </c>
       <c r="E29">
-        <v>225.1</v>
+        <v>237.1</v>
       </c>
       <c r="F29">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G29">
-        <v>5.5</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="30">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C30">
@@ -1152,13 +1152,13 @@
         <v>3.7</v>
       </c>
       <c r="E30">
-        <v>224.8</v>
+        <v>235.8</v>
       </c>
       <c r="F30">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="G30">
-        <v>5.5</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="31">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C31">
@@ -1177,13 +1177,13 @@
         <v>3.1</v>
       </c>
       <c r="E31">
-        <v>224.5</v>
+        <v>234.5</v>
       </c>
       <c r="F31">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="G31">
-        <v>5.5</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="32">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C32">
@@ -1202,13 +1202,13 @@
         <v>2.5</v>
       </c>
       <c r="E32">
-        <v>224.2</v>
+        <v>233.2</v>
       </c>
       <c r="F32">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="G32">
-        <v>5.5</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="33">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C33">
@@ -1227,13 +1227,13 @@
         <v>2.5</v>
       </c>
       <c r="E33">
-        <v>234.0</v>
+        <v>240.1</v>
       </c>
       <c r="F33">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="G33">
-        <v>8.9</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="34">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C34">
@@ -1252,13 +1252,13 @@
         <v>2.5</v>
       </c>
       <c r="E34">
-        <v>243.8</v>
+        <v>246.9</v>
       </c>
       <c r="F34">
         <v>3.7</v>
       </c>
       <c r="G34">
-        <v>12.2</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="35">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C35">
@@ -1277,13 +1277,13 @@
         <v>2.5</v>
       </c>
       <c r="E35">
-        <v>253.6</v>
+        <v>253.8</v>
       </c>
       <c r="F35">
         <v>3.8</v>
       </c>
       <c r="G35">
-        <v>15.6</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="36">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C36">
@@ -1302,13 +1302,13 @@
         <v>2.5</v>
       </c>
       <c r="E36">
-        <v>263.4</v>
+        <v>260.7</v>
       </c>
       <c r="F36">
-        <v>4.0</v>
+        <v>3.9</v>
       </c>
       <c r="G36">
-        <v>18.9</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="37">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C37">
@@ -1327,13 +1327,13 @@
         <v>2.5</v>
       </c>
       <c r="E37">
-        <v>273.1</v>
+        <v>267.5</v>
       </c>
       <c r="F37">
-        <v>4.1</v>
+        <v>4.0</v>
       </c>
       <c r="G37">
-        <v>22.2</v>
+        <v>16.6</v>
       </c>
     </row>
     <row r="38">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C38">
@@ -1352,13 +1352,13 @@
         <v>2.9</v>
       </c>
       <c r="E38">
-        <v>263.8</v>
+        <v>258.4</v>
       </c>
       <c r="F38">
-        <v>4.0</v>
+        <v>3.9</v>
       </c>
       <c r="G38">
-        <v>21.5</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="39">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C39">
@@ -1377,13 +1377,13 @@
         <v>3.3</v>
       </c>
       <c r="E39">
-        <v>254.5</v>
+        <v>249.3</v>
       </c>
       <c r="F39">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="G39">
-        <v>20.7</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="40">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C40">
@@ -1402,13 +1402,13 @@
         <v>3.6</v>
       </c>
       <c r="E40">
-        <v>245.2</v>
+        <v>240.2</v>
       </c>
       <c r="F40">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="G40">
-        <v>20.0</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="41">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C41">
@@ -1427,13 +1427,13 @@
         <v>4.0</v>
       </c>
       <c r="E41">
-        <v>235.9</v>
+        <v>231.0</v>
       </c>
       <c r="F41">
         <v>3.5</v>
       </c>
       <c r="G41">
-        <v>19.2</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="42">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C42">
@@ -1452,13 +1452,13 @@
         <v>4.4</v>
       </c>
       <c r="E42">
-        <v>226.6</v>
+        <v>221.9</v>
       </c>
       <c r="F42">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="G42">
-        <v>18.5</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="43">
@@ -1477,13 +1477,13 @@
         <v>4.0</v>
       </c>
       <c r="E43">
-        <v>221.7</v>
+        <v>218.0</v>
       </c>
       <c r="F43">
         <v>3.3</v>
       </c>
       <c r="G43">
-        <v>17.3</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="44">
@@ -1502,13 +1502,13 @@
         <v>3.5</v>
       </c>
       <c r="E44">
-        <v>216.8</v>
+        <v>214.1</v>
       </c>
       <c r="F44">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="G44">
-        <v>16.1</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="45">
@@ -1527,13 +1527,13 @@
         <v>3.1</v>
       </c>
       <c r="E45">
-        <v>212.0</v>
+        <v>210.1</v>
       </c>
       <c r="F45">
         <v>3.2</v>
       </c>
       <c r="G45">
-        <v>14.9</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="46">
@@ -1552,13 +1552,13 @@
         <v>2.6</v>
       </c>
       <c r="E46">
-        <v>207.1</v>
+        <v>206.2</v>
       </c>
       <c r="F46">
         <v>3.1</v>
       </c>
       <c r="G46">
-        <v>13.8</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="47">
@@ -3352,13 +3352,13 @@
         <v>7.5</v>
       </c>
       <c r="E118">
-        <v>206.9</v>
+        <v>206.1</v>
       </c>
       <c r="F118">
         <v>3.1</v>
       </c>
       <c r="G118">
-        <v>13.7</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="119">
@@ -3377,13 +3377,13 @@
         <v>6.5</v>
       </c>
       <c r="E119">
-        <v>209.2</v>
+        <v>207.4</v>
       </c>
       <c r="F119">
         <v>3.1</v>
       </c>
       <c r="G119">
-        <v>14.7</v>
+        <v>12.9</v>
       </c>
     </row>
     <row r="120">
@@ -3402,13 +3402,13 @@
         <v>5.6</v>
       </c>
       <c r="E120">
-        <v>211.4</v>
+        <v>208.7</v>
       </c>
       <c r="F120">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="G120">
-        <v>15.6</v>
+        <v>13.0</v>
       </c>
     </row>
     <row r="121">
@@ -3427,13 +3427,13 @@
         <v>4.6</v>
       </c>
       <c r="E121">
-        <v>213.6</v>
+        <v>210.0</v>
       </c>
       <c r="F121">
         <v>3.2</v>
       </c>
       <c r="G121">
-        <v>16.6</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="122">
@@ -3442,7 +3442,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C122">
@@ -3452,13 +3452,13 @@
         <v>3.7</v>
       </c>
       <c r="E122">
-        <v>215.8</v>
+        <v>211.3</v>
       </c>
       <c r="F122">
         <v>3.2</v>
       </c>
       <c r="G122">
-        <v>17.6</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="123">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C123">
@@ -3477,13 +3477,13 @@
         <v>3.7</v>
       </c>
       <c r="E123">
-        <v>226.4</v>
+        <v>221.8</v>
       </c>
       <c r="F123">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="G123">
-        <v>18.4</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="124">
@@ -3492,7 +3492,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C124">
@@ -3502,13 +3502,13 @@
         <v>3.7</v>
       </c>
       <c r="E124">
-        <v>237.1</v>
+        <v>232.2</v>
       </c>
       <c r="F124">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="G124">
-        <v>19.3</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="125">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C125">
@@ -3527,13 +3527,13 @@
         <v>3.8</v>
       </c>
       <c r="E125">
-        <v>247.8</v>
+        <v>242.7</v>
       </c>
       <c r="F125">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="G125">
-        <v>20.2</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="126">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C126">
@@ -3552,13 +3552,13 @@
         <v>3.8</v>
       </c>
       <c r="E126">
-        <v>258.5</v>
+        <v>253.1</v>
       </c>
       <c r="F126">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
       <c r="G126">
-        <v>21.1</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="127">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C127">
@@ -3577,13 +3577,13 @@
         <v>3.8</v>
       </c>
       <c r="E127">
-        <v>269.1</v>
+        <v>263.6</v>
       </c>
       <c r="F127">
         <v>4.0</v>
       </c>
       <c r="G127">
-        <v>21.9</v>
+        <v>16.4</v>
       </c>
     </row>
     <row r="128">
@@ -3592,7 +3592,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C128">
@@ -3602,13 +3602,13 @@
         <v>4.3</v>
       </c>
       <c r="E128">
-        <v>260.5</v>
+        <v>257.9</v>
       </c>
       <c r="F128">
         <v>3.9</v>
       </c>
       <c r="G128">
-        <v>18.6</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="129">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C129">
@@ -3627,13 +3627,13 @@
         <v>4.9</v>
       </c>
       <c r="E129">
-        <v>251.9</v>
+        <v>252.2</v>
       </c>
       <c r="F129">
         <v>3.8</v>
       </c>
       <c r="G129">
-        <v>15.4</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="130">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C130">
@@ -3652,13 +3652,13 @@
         <v>5.4</v>
       </c>
       <c r="E130">
-        <v>243.2</v>
+        <v>246.4</v>
       </c>
       <c r="F130">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="G130">
-        <v>12.1</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="131">
@@ -3667,7 +3667,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>HAZ</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C131">
@@ -3677,13 +3677,13 @@
         <v>6.0</v>
       </c>
       <c r="E131">
-        <v>234.6</v>
+        <v>240.7</v>
       </c>
       <c r="F131">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="G131">
-        <v>8.8</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="132">
@@ -3692,7 +3692,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>FZ</t>
         </is>
       </c>
       <c r="C132">
@@ -3702,13 +3702,13 @@
         <v>6.5</v>
       </c>
       <c r="E132">
-        <v>225.9</v>
+        <v>235.0</v>
       </c>
       <c r="F132">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="G132">
-        <v>5.5</v>
+        <v>14.6</v>
       </c>
     </row>
     <row r="133">
@@ -3717,7 +3717,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C133">
@@ -3727,13 +3727,13 @@
         <v>5.7</v>
       </c>
       <c r="E133">
-        <v>225.6</v>
+        <v>235.6</v>
       </c>
       <c r="F133">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="G133">
-        <v>5.5</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="134">
@@ -3742,7 +3742,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C134">
@@ -3752,13 +3752,13 @@
         <v>5.0</v>
       </c>
       <c r="E134">
-        <v>225.2</v>
+        <v>236.2</v>
       </c>
       <c r="F134">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="G134">
-        <v>5.5</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="135">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C135">
@@ -3777,13 +3777,13 @@
         <v>4.2</v>
       </c>
       <c r="E135">
-        <v>224.9</v>
+        <v>236.9</v>
       </c>
       <c r="F135">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G135">
-        <v>5.5</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="136">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C136">
@@ -3802,13 +3802,13 @@
         <v>3.5</v>
       </c>
       <c r="E136">
-        <v>224.6</v>
+        <v>237.5</v>
       </c>
       <c r="F136">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G136">
-        <v>5.5</v>
+        <v>18.4</v>
       </c>
     </row>
     <row r="137">
@@ -3817,7 +3817,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C137">
@@ -3827,13 +3827,13 @@
         <v>2.7</v>
       </c>
       <c r="E137">
-        <v>224.2</v>
+        <v>238.1</v>
       </c>
       <c r="F137">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G137">
-        <v>5.5</v>
+        <v>19.4</v>
       </c>
     </row>
     <row r="138">
@@ -3842,7 +3842,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C138">
@@ -3852,13 +3852,13 @@
         <v>2.7</v>
       </c>
       <c r="E138">
-        <v>225.0</v>
+        <v>239.0</v>
       </c>
       <c r="F138">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G138">
-        <v>5.5</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="139">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C139">
@@ -3877,13 +3877,13 @@
         <v>2.7</v>
       </c>
       <c r="E139">
-        <v>225.9</v>
+        <v>239.9</v>
       </c>
       <c r="F139">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G139">
-        <v>5.5</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="140">
@@ -3892,7 +3892,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C140">
@@ -3902,13 +3902,13 @@
         <v>2.6</v>
       </c>
       <c r="E140">
-        <v>226.7</v>
+        <v>240.8</v>
       </c>
       <c r="F140">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G140">
-        <v>5.6</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="141">
@@ -3917,7 +3917,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C141">
@@ -3927,13 +3927,13 @@
         <v>2.6</v>
       </c>
       <c r="E141">
-        <v>227.6</v>
+        <v>241.7</v>
       </c>
       <c r="F141">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G141">
-        <v>5.6</v>
+        <v>19.7</v>
       </c>
     </row>
     <row r="142">
@@ -3942,7 +3942,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C142">
@@ -3952,13 +3952,13 @@
         <v>2.6</v>
       </c>
       <c r="E142">
-        <v>228.4</v>
+        <v>242.6</v>
       </c>
       <c r="F142">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G142">
-        <v>5.6</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="143">
@@ -3967,7 +3967,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C143">
@@ -3977,13 +3977,13 @@
         <v>3.3</v>
       </c>
       <c r="E143">
-        <v>228.5</v>
+        <v>242.7</v>
       </c>
       <c r="F143">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G143">
-        <v>5.6</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="144">
@@ -3992,7 +3992,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C144">
@@ -4002,13 +4002,13 @@
         <v>4.0</v>
       </c>
       <c r="E144">
-        <v>228.7</v>
+        <v>242.8</v>
       </c>
       <c r="F144">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G144">
-        <v>5.6</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="145">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C145">
@@ -4027,13 +4027,13 @@
         <v>4.7</v>
       </c>
       <c r="E145">
-        <v>228.8</v>
+        <v>242.9</v>
       </c>
       <c r="F145">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G145">
-        <v>5.6</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="146">
@@ -4042,7 +4042,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C146">
@@ -4052,13 +4052,13 @@
         <v>5.4</v>
       </c>
       <c r="E146">
-        <v>228.9</v>
+        <v>243.1</v>
       </c>
       <c r="F146">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G146">
-        <v>5.6</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="147">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C147">
@@ -4077,13 +4077,13 @@
         <v>6.1</v>
       </c>
       <c r="E147">
-        <v>229.0</v>
+        <v>243.2</v>
       </c>
       <c r="F147">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G147">
-        <v>5.6</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="148">
@@ -4092,7 +4092,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C148">
@@ -4102,13 +4102,13 @@
         <v>5.8</v>
       </c>
       <c r="E148">
-        <v>227.6</v>
+        <v>241.7</v>
       </c>
       <c r="F148">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G148">
-        <v>5.6</v>
+        <v>19.7</v>
       </c>
     </row>
     <row r="149">
@@ -4117,7 +4117,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C149">
@@ -4127,13 +4127,13 @@
         <v>5.6</v>
       </c>
       <c r="E149">
-        <v>226.2</v>
+        <v>240.2</v>
       </c>
       <c r="F149">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G149">
-        <v>5.6</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="150">
@@ -4142,7 +4142,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C150">
@@ -4152,13 +4152,13 @@
         <v>5.3</v>
       </c>
       <c r="E150">
-        <v>224.8</v>
+        <v>238.7</v>
       </c>
       <c r="F150">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G150">
-        <v>5.5</v>
+        <v>19.4</v>
       </c>
     </row>
     <row r="151">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C151">
@@ -4177,13 +4177,13 @@
         <v>5.1</v>
       </c>
       <c r="E151">
-        <v>223.4</v>
+        <v>237.2</v>
       </c>
       <c r="F151">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="G151">
-        <v>5.5</v>
+        <v>19.3</v>
       </c>
     </row>
     <row r="152">
@@ -4192,7 +4192,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C152">
@@ -4202,13 +4202,13 @@
         <v>4.8</v>
       </c>
       <c r="E152">
-        <v>221.9</v>
+        <v>235.7</v>
       </c>
       <c r="F152">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="G152">
-        <v>5.4</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="153">
@@ -4217,7 +4217,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C153">
@@ -4227,13 +4227,13 @@
         <v>4.4</v>
       </c>
       <c r="E153">
-        <v>221.1</v>
+        <v>234.8</v>
       </c>
       <c r="F153">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="G153">
-        <v>5.4</v>
+        <v>19.1</v>
       </c>
     </row>
     <row r="154">
@@ -4242,7 +4242,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C154">
@@ -4252,13 +4252,13 @@
         <v>3.9</v>
       </c>
       <c r="E154">
-        <v>220.3</v>
+        <v>234.0</v>
       </c>
       <c r="F154">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="G154">
-        <v>5.4</v>
+        <v>19.1</v>
       </c>
     </row>
     <row r="155">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C155">
@@ -4277,13 +4277,13 @@
         <v>3.5</v>
       </c>
       <c r="E155">
-        <v>219.5</v>
+        <v>233.2</v>
       </c>
       <c r="F155">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="G155">
-        <v>5.4</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="156">
@@ -4292,7 +4292,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C156">
@@ -4302,13 +4302,13 @@
         <v>3.0</v>
       </c>
       <c r="E156">
-        <v>218.7</v>
+        <v>232.3</v>
       </c>
       <c r="F156">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="G156">
-        <v>5.4</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="157">
@@ -4317,7 +4317,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="C157">
@@ -4327,13 +4327,13 @@
         <v>2.6</v>
       </c>
       <c r="E157">
-        <v>217.9</v>
+        <v>231.5</v>
       </c>
       <c r="F157">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="G157">
-        <v>5.3</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="158">
@@ -4352,13 +4352,13 @@
         <v>2.9</v>
       </c>
       <c r="E158">
-        <v>218.7</v>
+        <v>229.5</v>
       </c>
       <c r="F158">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="G158">
-        <v>5.4</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="159">
@@ -4377,13 +4377,13 @@
         <v>3.1</v>
       </c>
       <c r="E159">
-        <v>219.4</v>
+        <v>227.5</v>
       </c>
       <c r="F159">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="G159">
-        <v>5.4</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="160">
@@ -4402,13 +4402,13 @@
         <v>3.4</v>
       </c>
       <c r="E160">
-        <v>220.2</v>
+        <v>225.6</v>
       </c>
       <c r="F160">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="G160">
-        <v>5.4</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="161">
@@ -4427,13 +4427,13 @@
         <v>3.6</v>
       </c>
       <c r="E161">
-        <v>220.9</v>
+        <v>223.6</v>
       </c>
       <c r="F161">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="G161">
-        <v>5.4</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="162">
@@ -4513,44 +4513,44 @@
         </is>
       </c>
       <c r="B2">
-        <v>214.6</v>
+        <v>215.7</v>
       </c>
       <c r="C2">
+        <v>1.4</v>
+      </c>
+      <c r="D2">
+        <v>226.6</v>
+      </c>
+      <c r="E2">
+        <v>3.4</v>
+      </c>
+      <c r="F2">
+        <v>10.9</v>
+      </c>
+      <c r="G2">
         <v>5.0</v>
-      </c>
-      <c r="D2">
-        <v>220.0</v>
-      </c>
-      <c r="E2">
-        <v>5.0</v>
-      </c>
-      <c r="F2">
-        <v>5.4</v>
-      </c>
-      <c r="G2">
-        <v>2.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fusion Zone (E9018)</t>
+          <t>Weld (Fusion Zone)</t>
         </is>
       </c>
       <c r="B3">
-        <v>196.0</v>
+        <v>200.2</v>
       </c>
       <c r="C3">
-        <v>5.7</v>
+        <v>16.4</v>
       </c>
       <c r="D3">
-        <v>209.0</v>
+        <v>213.5</v>
       </c>
       <c r="E3">
-        <v>5.7</v>
+        <v>3.2</v>
       </c>
       <c r="F3">
-        <v>13.0</v>
+        <v>13.3</v>
       </c>
       <c r="G3">
         <v>6.6</v>
@@ -4559,26 +4559,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HAZ (CGHAZ)</t>
+          <t>HAZ</t>
         </is>
       </c>
       <c r="B4">
-        <v>252.6</v>
+        <v>218.6</v>
       </c>
       <c r="C4">
-        <v>7.0</v>
+        <v>3.1</v>
       </c>
       <c r="D4">
-        <v>275.0</v>
+        <v>237.6</v>
       </c>
       <c r="E4">
-        <v>7.0</v>
+        <v>3.6</v>
       </c>
       <c r="F4">
-        <v>22.4</v>
+        <v>19.0</v>
       </c>
       <c r="G4">
-        <v>8.9</v>
+        <v>8.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>